<commit_message>
fixed colors in sankey diagram by remocing spaces that stop double coding for S-AS situations.
</commit_message>
<xml_diff>
--- a/Data/Sankey_diagram_table.xlsx
+++ b/Data/Sankey_diagram_table.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexbl/Desktop/MarEEchange/1_Paper_publi/1_SES/R/prOACT_pathways/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59BD3776-D525-774D-85AD-5F95E6190A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CC6E6A0-0876-E449-A1C3-0FD0C735DD3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="660" windowWidth="15120" windowHeight="17900" activeTab="1" xr2:uid="{714A1C6C-974B-1E4A-9034-5DDE98B770F7}"/>
+    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{714A1C6C-974B-1E4A-9034-5DDE98B770F7}"/>
   </bookViews>
   <sheets>
-    <sheet name="Submission_2" sheetId="2" r:id="rId1"/>
-    <sheet name="Submission_1" sheetId="1" r:id="rId2"/>
+    <sheet name="Sankey" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Submission_1!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sankey!$A$1:$C$1</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="38">
   <si>
     <t>Objectives</t>
   </si>
@@ -151,23 +150,19 @@
   </si>
   <si>
     <t>Measures</t>
+  </si>
+  <si>
+    <t>SE_AS_recreational</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -193,9 +188,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -530,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1BD5AB6-4321-1D48-9ECA-644E93EAEEF8}">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.1640625" bestFit="1" customWidth="1"/>
@@ -1869,519 +1863,74 @@
         <v>24</v>
       </c>
     </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A122" t="s">
+        <v>19</v>
+      </c>
+      <c r="B122" t="s">
+        <v>37</v>
+      </c>
+      <c r="C122" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A123" t="s">
+        <v>19</v>
+      </c>
+      <c r="B123" t="s">
+        <v>37</v>
+      </c>
+      <c r="C123" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A124" t="s">
+        <v>4</v>
+      </c>
+      <c r="B124" t="s">
+        <v>37</v>
+      </c>
+      <c r="C124" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A125" t="s">
+        <v>4</v>
+      </c>
+      <c r="B125" t="s">
+        <v>37</v>
+      </c>
+      <c r="C125" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A126" t="s">
+        <v>7</v>
+      </c>
+      <c r="B126" t="s">
+        <v>37</v>
+      </c>
+      <c r="C126" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A127" t="s">
+        <v>7</v>
+      </c>
+      <c r="B127" t="s">
+        <v>37</v>
+      </c>
+      <c r="C127" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:C1" xr:uid="{B1BD5AB6-4321-1D48-9ECA-644E93EAEEF8}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74B3850C-E65A-1944-A60F-6755105C59A4}">
-  <dimension ref="A1:C45"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="29.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" t="s">
-        <v>3</v>
-      </c>
-      <c r="C12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C19" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>28</v>
-      </c>
-      <c r="B21" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>28</v>
-      </c>
-      <c r="B23" t="s">
-        <v>5</v>
-      </c>
-      <c r="C23" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>27</v>
-      </c>
-      <c r="B24" t="s">
-        <v>3</v>
-      </c>
-      <c r="C24" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25" t="s">
-        <v>19</v>
-      </c>
-      <c r="C25" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" t="s">
-        <v>5</v>
-      </c>
-      <c r="C26" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27" t="s">
-        <v>3</v>
-      </c>
-      <c r="C27" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>26</v>
-      </c>
-      <c r="B28" t="s">
-        <v>13</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>26</v>
-      </c>
-      <c r="B29" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>26</v>
-      </c>
-      <c r="B30" t="s">
-        <v>22</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>26</v>
-      </c>
-      <c r="B31" t="s">
-        <v>15</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>26</v>
-      </c>
-      <c r="B32" t="s">
-        <v>11</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>26</v>
-      </c>
-      <c r="B33" t="s">
-        <v>5</v>
-      </c>
-      <c r="C33" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>26</v>
-      </c>
-      <c r="B34" t="s">
-        <v>14</v>
-      </c>
-      <c r="C34" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>29</v>
-      </c>
-      <c r="B35" t="s">
-        <v>3</v>
-      </c>
-      <c r="C35" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>29</v>
-      </c>
-      <c r="B36" t="s">
-        <v>20</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>29</v>
-      </c>
-      <c r="B37" t="s">
-        <v>8</v>
-      </c>
-      <c r="C37" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
-        <v>29</v>
-      </c>
-      <c r="B38" t="s">
-        <v>22</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
-        <v>29</v>
-      </c>
-      <c r="B39" t="s">
-        <v>5</v>
-      </c>
-      <c r="C39" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>29</v>
-      </c>
-      <c r="B40" t="s">
-        <v>21</v>
-      </c>
-      <c r="C40" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>29</v>
-      </c>
-      <c r="B41" t="s">
-        <v>14</v>
-      </c>
-      <c r="C41" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>30</v>
-      </c>
-      <c r="B42" t="s">
-        <v>3</v>
-      </c>
-      <c r="C42" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>30</v>
-      </c>
-      <c r="B43" t="s">
-        <v>12</v>
-      </c>
-      <c r="C43" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>30</v>
-      </c>
-      <c r="B44" t="s">
-        <v>10</v>
-      </c>
-      <c r="C44" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>30</v>
-      </c>
-      <c r="B45" t="s">
-        <v>5</v>
-      </c>
-      <c r="C45" t="s">
-        <v>31</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
created new Sankey figure.
</commit_message>
<xml_diff>
--- a/Data/Sankey_diagram_table.xlsx
+++ b/Data/Sankey_diagram_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexbl/Desktop/MarEEchange/1_Paper_publi/1_SES/R/prOACT_pathways/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CC6E6A0-0876-E449-A1C3-0FD0C735DD3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6138FE91-27B6-134F-9EA4-30ECBED73E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{714A1C6C-974B-1E4A-9034-5DDE98B770F7}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="38">
   <si>
     <t>Objectives</t>
   </si>
@@ -524,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1BD5AB6-4321-1D48-9ECA-644E93EAEEF8}">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.1640625" bestFit="1" customWidth="1"/>
@@ -1458,13 +1458,13 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B85" t="s">
         <v>32</v>
       </c>
       <c r="C85" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.2">
@@ -1475,7 +1475,7 @@
         <v>32</v>
       </c>
       <c r="C86" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.2">
@@ -1486,7 +1486,7 @@
         <v>32</v>
       </c>
       <c r="C87" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.2">
@@ -1497,7 +1497,7 @@
         <v>32</v>
       </c>
       <c r="C88" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.2">
@@ -1508,7 +1508,7 @@
         <v>32</v>
       </c>
       <c r="C89" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
@@ -1519,7 +1519,7 @@
         <v>32</v>
       </c>
       <c r="C90" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.2">
@@ -1530,18 +1530,18 @@
         <v>32</v>
       </c>
       <c r="C91" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B92" t="s">
         <v>32</v>
       </c>
       <c r="C92" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.2">
@@ -1552,7 +1552,7 @@
         <v>32</v>
       </c>
       <c r="C93" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.2">
@@ -1563,7 +1563,7 @@
         <v>32</v>
       </c>
       <c r="C94" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.2">
@@ -1574,7 +1574,7 @@
         <v>32</v>
       </c>
       <c r="C95" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
@@ -1585,7 +1585,7 @@
         <v>32</v>
       </c>
       <c r="C96" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.2">
@@ -1596,7 +1596,7 @@
         <v>32</v>
       </c>
       <c r="C97" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.2">
@@ -1607,18 +1607,18 @@
         <v>32</v>
       </c>
       <c r="C98" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B99" t="s">
         <v>32</v>
       </c>
       <c r="C99" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.2">
@@ -1629,7 +1629,7 @@
         <v>32</v>
       </c>
       <c r="C100" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.2">
@@ -1640,7 +1640,7 @@
         <v>32</v>
       </c>
       <c r="C101" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.2">
@@ -1651,7 +1651,7 @@
         <v>32</v>
       </c>
       <c r="C102" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.2">
@@ -1662,7 +1662,7 @@
         <v>32</v>
       </c>
       <c r="C103" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.2">
@@ -1673,7 +1673,7 @@
         <v>32</v>
       </c>
       <c r="C104" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.2">
@@ -1684,18 +1684,18 @@
         <v>32</v>
       </c>
       <c r="C105" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B106" t="s">
         <v>32</v>
       </c>
       <c r="C106" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
@@ -1706,7 +1706,7 @@
         <v>32</v>
       </c>
       <c r="C107" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
@@ -1717,7 +1717,7 @@
         <v>32</v>
       </c>
       <c r="C108" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.2">
@@ -1728,7 +1728,7 @@
         <v>32</v>
       </c>
       <c r="C109" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.2">
@@ -1739,7 +1739,7 @@
         <v>32</v>
       </c>
       <c r="C110" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.2">
@@ -1750,7 +1750,7 @@
         <v>32</v>
       </c>
       <c r="C111" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.2">
@@ -1761,18 +1761,18 @@
         <v>32</v>
       </c>
       <c r="C112" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B113" t="s">
         <v>32</v>
       </c>
       <c r="C113" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.2">
@@ -1783,7 +1783,7 @@
         <v>32</v>
       </c>
       <c r="C114" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.2">
@@ -1794,7 +1794,7 @@
         <v>32</v>
       </c>
       <c r="C115" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.2">
@@ -1805,7 +1805,7 @@
         <v>32</v>
       </c>
       <c r="C116" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.2">
@@ -1816,7 +1816,7 @@
         <v>32</v>
       </c>
       <c r="C117" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.2">
@@ -1827,7 +1827,7 @@
         <v>32</v>
       </c>
       <c r="C118" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.2">
@@ -1838,15 +1838,15 @@
         <v>32</v>
       </c>
       <c r="C119" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B120" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C120" t="s">
         <v>25</v>
@@ -1860,15 +1860,15 @@
         <v>33</v>
       </c>
       <c r="C121" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B122" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C122" t="s">
         <v>24</v>
@@ -1882,18 +1882,18 @@
         <v>37</v>
       </c>
       <c r="C123" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B124" t="s">
         <v>37</v>
       </c>
       <c r="C124" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.2">
@@ -1904,18 +1904,18 @@
         <v>37</v>
       </c>
       <c r="C125" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B126" t="s">
         <v>37</v>
       </c>
       <c r="C126" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.2">
@@ -1926,6 +1926,17 @@
         <v>37</v>
       </c>
       <c r="C127" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A128" t="s">
+        <v>7</v>
+      </c>
+      <c r="B128" t="s">
+        <v>37</v>
+      </c>
+      <c r="C128" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>